<commit_message>
interlab variance analysis and Sirius annotation
</commit_message>
<xml_diff>
--- a/3_annotation_manual/HE/2_combine_annotation/consensus_lab_annotations.xlsx
+++ b/3_annotation_manual/HE/2_combine_annotation/consensus_lab_annotations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scientificnet-my.sharepoint.com/personal/plouail_eurac_edu/Documents/Documents/GitHub/HUMAN_Ring_Trial/3_annotation_manual/HE/2_combine_annotation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_B99231273CB960E208153C8CD35E02E94258ED34" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9CBC8A5-4D22-4995-9AD9-91D6C798D925}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_B99231273CB960E208153C8CD35E02E94258ED34" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1CFF6E6-D326-4472-B283-51B8E1054976}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2244,6 +2244,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2529,7 +2533,12 @@
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="10" max="10" width="35.33203125" customWidth="1"/>
+    <col min="11" max="11" width="27.21875" customWidth="1"/>
     <col min="12" max="12" width="56.109375" customWidth="1"/>
+    <col min="18" max="18" width="27.77734375" customWidth="1"/>
+    <col min="19" max="19" width="22.44140625" customWidth="1"/>
+    <col min="20" max="20" width="32.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">

</xml_diff>